<commit_message>
protein accouting bug fix
</commit_message>
<xml_diff>
--- a/tests/data/cattle/output/excel/cattle.xlsx
+++ b/tests/data/cattle/output/excel/cattle.xlsx
@@ -477,16 +477,16 @@
         <v>2030</v>
       </c>
       <c r="B3" t="n">
-        <v>4503509.251804466</v>
+        <v>3951689.846485116</v>
       </c>
       <c r="C3" t="n">
-        <v>924927.1488617986</v>
+        <v>1489542.593964852</v>
       </c>
       <c r="D3" t="n">
-        <v>5428436.400666265</v>
+        <v>5441232.440449968</v>
       </c>
       <c r="E3" t="n">
-        <v>4.869042126557121</v>
+        <v>2.652955251159713</v>
       </c>
     </row>
     <row r="4">
@@ -494,16 +494,16 @@
         <v>2040</v>
       </c>
       <c r="B4" t="n">
-        <v>785088.7318133655</v>
+        <v>1036975.803072285</v>
       </c>
       <c r="C4" t="n">
-        <v>4031022.485568935</v>
+        <v>3773294.450846681</v>
       </c>
       <c r="D4" t="n">
-        <v>4816111.2173823</v>
+        <v>4810270.253918966</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1947616850622848</v>
+        <v>0.2748197408340609</v>
       </c>
     </row>
     <row r="5">

</xml_diff>